<commit_message>
GBDS APRIL FILES 2026 | fliqlo@GBDS
</commit_message>
<xml_diff>
--- a/GBDS APRIL FILES 2026/CSR MONTH OF APRIL 2026.xlsx
+++ b/GBDS APRIL FILES 2026/CSR MONTH OF APRIL 2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\GBDS APRIL FILES 2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27592F88-EE38-4265-82EE-E3B0ABCB5548}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1B1C456-FE6E-488E-B50E-3EA788F360EE}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="8" activeTab="20" xr2:uid="{67C3A74A-A57E-4AB5-8CD3-31B592A14032}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{67C3A74A-A57E-4AB5-8CD3-31B592A14032}"/>
   </bookViews>
   <sheets>
     <sheet name="CSR | APRIL" sheetId="902" r:id="rId1"/>
@@ -23,13 +23,13 @@
     <sheet name="04-02 R2" sheetId="1550" r:id="rId8"/>
     <sheet name="04-02 R3" sheetId="1551" r:id="rId9"/>
     <sheet name="(3)" sheetId="1552" r:id="rId10"/>
-    <sheet name="04-03 R1" sheetId="1553" r:id="rId11"/>
-    <sheet name="04-03 R2" sheetId="1554" r:id="rId12"/>
-    <sheet name="04-03 R3" sheetId="1555" r:id="rId13"/>
+    <sheet name="04-03 R1 HOLIDAY" sheetId="1553" r:id="rId11"/>
+    <sheet name="04-03 R2 HOLIDAY" sheetId="1554" r:id="rId12"/>
+    <sheet name="04-03 R3 HOLIDAY" sheetId="1555" r:id="rId13"/>
     <sheet name="(4)" sheetId="1556" r:id="rId14"/>
-    <sheet name="04-04 R1" sheetId="1557" r:id="rId15"/>
-    <sheet name="04-04 R2" sheetId="1558" r:id="rId16"/>
-    <sheet name="04-04 R3" sheetId="1559" r:id="rId17"/>
+    <sheet name="04-04 R1 HOLIDAY" sheetId="1557" r:id="rId15"/>
+    <sheet name="04-04 R2 HOLIDAY" sheetId="1558" r:id="rId16"/>
+    <sheet name="04-04 R3 HOLIDAY" sheetId="1559" r:id="rId17"/>
     <sheet name="(6)" sheetId="1560" r:id="rId18"/>
     <sheet name="04-06R1" sheetId="1561" r:id="rId19"/>
     <sheet name="04-06 R2" sheetId="1562" r:id="rId20"/>
@@ -50,12 +50,12 @@
     <definedName name="_xlnm.Print_Area" localSheetId="6">'04-02 R1'!$A$1:$Z$43</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="7">'04-02 R2'!$A$1:$V$44</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="8">'04-02 R3'!$A$1:$V$44</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="10">'04-03 R1'!$A$1:$Z$43</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="11">'04-03 R2'!$A$1:$V$44</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="12">'04-03 R3'!$A$1:$V$44</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="14">'04-04 R1'!$A$1:$Z$43</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="15">'04-04 R2'!$A$1:$V$44</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="16">'04-04 R3'!$A$1:$V$44</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="10">'04-03 R1 HOLIDAY'!$A$1:$Z$43</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="11">'04-03 R2 HOLIDAY'!$A$1:$V$44</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="12">'04-03 R3 HOLIDAY'!$A$1:$V$44</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="14">'04-04 R1 HOLIDAY'!$A$1:$Z$43</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="15">'04-04 R2 HOLIDAY'!$A$1:$V$44</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="16">'04-04 R3 HOLIDAY'!$A$1:$V$44</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="19">'04-06 R2'!$A$1:$V$44</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="20">'04-06 R3'!$A$1:$V$44</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="18">'04-06R1'!$A$1:$Z$43</definedName>
@@ -76,7 +76,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1765" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1783" uniqueCount="87">
   <si>
     <t>CHECKER STOCK REPORT</t>
   </si>
@@ -301,6 +301,42 @@
   </si>
   <si>
     <t>DATE ___________04/06/2026___________</t>
+  </si>
+  <si>
+    <t>18/20B</t>
+  </si>
+  <si>
+    <t>8/4B</t>
+  </si>
+  <si>
+    <t>2/12B</t>
+  </si>
+  <si>
+    <t>6/4B</t>
+  </si>
+  <si>
+    <t>16B</t>
+  </si>
+  <si>
+    <t>6/20B</t>
+  </si>
+  <si>
+    <t>1/19B</t>
+  </si>
+  <si>
+    <t>3/12B</t>
+  </si>
+  <si>
+    <t>3/4B</t>
+  </si>
+  <si>
+    <t>21/22B</t>
+  </si>
+  <si>
+    <t>7/3B</t>
+  </si>
+  <si>
+    <t>29/1B</t>
   </si>
 </sst>
 </file>
@@ -22762,7 +22798,8 @@
   <cols>
     <col min="1" max="1" width="1.140625" style="2" customWidth="1"/>
     <col min="2" max="2" width="14.42578125" style="2" customWidth="1"/>
-    <col min="3" max="8" width="5.7109375" style="2" customWidth="1"/>
+    <col min="3" max="7" width="5.7109375" style="2" customWidth="1"/>
+    <col min="8" max="8" width="7" style="2" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="8" style="2" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="7" style="2" bestFit="1" customWidth="1"/>
     <col min="11" max="13" width="5.7109375" style="2" customWidth="1"/>
@@ -23131,12 +23168,16 @@
     </row>
     <row r="8" spans="2:27" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="12"/>
-      <c r="C8" s="13"/>
+      <c r="C8" s="13">
+        <v>2</v>
+      </c>
       <c r="D8" s="14"/>
       <c r="E8" s="14"/>
       <c r="F8" s="14"/>
       <c r="G8" s="14"/>
-      <c r="H8" s="14"/>
+      <c r="H8" s="14">
+        <v>27</v>
+      </c>
       <c r="I8" s="14"/>
       <c r="J8" s="14"/>
       <c r="K8" s="14"/>
@@ -23148,10 +23189,14 @@
       <c r="Q8" s="14"/>
       <c r="R8" s="14"/>
       <c r="S8" s="14"/>
-      <c r="T8" s="14"/>
+      <c r="T8" s="14">
+        <v>1</v>
+      </c>
       <c r="U8" s="14"/>
       <c r="V8" s="14"/>
-      <c r="W8" s="14"/>
+      <c r="W8" s="14">
+        <v>1</v>
+      </c>
       <c r="X8" s="59"/>
       <c r="Y8" s="15"/>
     </row>
@@ -23319,12 +23364,16 @@
       <c r="B15" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="22"/>
+      <c r="C15" s="22">
+        <v>1</v>
+      </c>
       <c r="D15" s="23"/>
       <c r="E15" s="23"/>
       <c r="F15" s="23"/>
       <c r="G15" s="23"/>
-      <c r="H15" s="23"/>
+      <c r="H15" s="23" t="s">
+        <v>75</v>
+      </c>
       <c r="I15" s="23"/>
       <c r="J15" s="23"/>
       <c r="K15" s="23"/>
@@ -23336,10 +23385,14 @@
       <c r="Q15" s="23"/>
       <c r="R15" s="23"/>
       <c r="S15" s="23"/>
-      <c r="T15" s="23"/>
+      <c r="T15" s="23">
+        <v>0</v>
+      </c>
       <c r="U15" s="23"/>
       <c r="V15" s="23"/>
-      <c r="W15" s="23"/>
+      <c r="W15" s="23">
+        <v>0</v>
+      </c>
       <c r="X15" s="61"/>
       <c r="Y15" s="24"/>
     </row>
@@ -23347,12 +23400,16 @@
       <c r="B16" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="C16" s="57"/>
+      <c r="C16" s="57">
+        <v>1</v>
+      </c>
       <c r="D16" s="58"/>
       <c r="E16" s="27"/>
       <c r="F16" s="27"/>
       <c r="G16" s="28"/>
-      <c r="H16" s="28"/>
+      <c r="H16" s="28" t="s">
+        <v>76</v>
+      </c>
       <c r="I16" s="28"/>
       <c r="J16" s="28"/>
       <c r="K16" s="56"/>
@@ -23364,10 +23421,14 @@
       <c r="Q16" s="28"/>
       <c r="R16" s="28"/>
       <c r="S16" s="28"/>
-      <c r="T16" s="28"/>
+      <c r="T16" s="28">
+        <v>1</v>
+      </c>
       <c r="U16" s="28"/>
       <c r="V16" s="28"/>
-      <c r="W16" s="56"/>
+      <c r="W16" s="56">
+        <v>1</v>
+      </c>
       <c r="X16" s="62"/>
       <c r="Y16" s="29"/>
     </row>
@@ -23771,17 +23832,27 @@
       <c r="C24" s="13"/>
       <c r="D24" s="14"/>
       <c r="E24" s="14"/>
-      <c r="F24" s="14"/>
+      <c r="F24" s="14">
+        <v>1</v>
+      </c>
       <c r="G24" s="14"/>
-      <c r="H24" s="14"/>
+      <c r="H24" s="14">
+        <v>71</v>
+      </c>
       <c r="I24" s="14"/>
       <c r="J24" s="14"/>
       <c r="K24" s="14"/>
-      <c r="L24" s="14"/>
-      <c r="M24" s="14"/>
+      <c r="L24" s="14">
+        <v>10</v>
+      </c>
+      <c r="M24" s="14">
+        <v>695</v>
+      </c>
       <c r="N24" s="14"/>
       <c r="O24" s="14"/>
-      <c r="P24" s="14"/>
+      <c r="P24" s="14">
+        <v>5</v>
+      </c>
       <c r="Q24" s="14"/>
       <c r="R24" s="14"/>
       <c r="S24" s="14"/>
@@ -23957,17 +24028,27 @@
       <c r="C31" s="22"/>
       <c r="D31" s="23"/>
       <c r="E31" s="23"/>
-      <c r="F31" s="23"/>
+      <c r="F31" s="23">
+        <v>0</v>
+      </c>
       <c r="G31" s="23"/>
-      <c r="H31" s="23"/>
+      <c r="H31" s="23">
+        <v>0</v>
+      </c>
       <c r="I31" s="23"/>
       <c r="J31" s="23"/>
       <c r="K31" s="23"/>
-      <c r="L31" s="23"/>
-      <c r="M31" s="23"/>
+      <c r="L31" s="23">
+        <v>7</v>
+      </c>
+      <c r="M31" s="23">
+        <v>51</v>
+      </c>
       <c r="N31" s="23"/>
       <c r="O31" s="23"/>
-      <c r="P31" s="23"/>
+      <c r="P31" s="23">
+        <v>0</v>
+      </c>
       <c r="Q31" s="23"/>
       <c r="R31" s="23"/>
       <c r="S31" s="23"/>
@@ -23985,17 +24066,27 @@
       <c r="C32" s="26"/>
       <c r="D32" s="27"/>
       <c r="E32" s="27"/>
-      <c r="F32" s="27"/>
+      <c r="F32" s="27">
+        <v>1</v>
+      </c>
       <c r="G32" s="28"/>
-      <c r="H32" s="28"/>
+      <c r="H32" s="28">
+        <v>71</v>
+      </c>
       <c r="I32" s="28"/>
       <c r="J32" s="28"/>
       <c r="K32" s="28"/>
-      <c r="L32" s="28"/>
-      <c r="M32" s="28"/>
+      <c r="L32" s="28">
+        <v>3</v>
+      </c>
+      <c r="M32" s="28">
+        <v>644</v>
+      </c>
       <c r="N32" s="28"/>
       <c r="O32" s="23"/>
-      <c r="P32" s="28"/>
+      <c r="P32" s="28">
+        <v>5</v>
+      </c>
       <c r="Q32" s="28"/>
       <c r="R32" s="28"/>
       <c r="S32" s="28"/>
@@ -24135,16 +24226,32 @@
       <c r="C36" s="46"/>
       <c r="D36" s="41"/>
       <c r="E36" s="42"/>
-      <c r="F36" s="42"/>
-      <c r="G36" s="42"/>
-      <c r="H36" s="42"/>
-      <c r="I36" s="42"/>
-      <c r="J36" s="42"/>
-      <c r="K36" s="42"/>
-      <c r="L36" s="42"/>
+      <c r="F36" s="42">
+        <v>682</v>
+      </c>
+      <c r="G36" s="42">
+        <v>21</v>
+      </c>
+      <c r="H36" s="42">
+        <v>5</v>
+      </c>
+      <c r="I36" s="42">
+        <v>9</v>
+      </c>
+      <c r="J36" s="42">
+        <v>3</v>
+      </c>
+      <c r="K36" s="42">
+        <v>11</v>
+      </c>
+      <c r="L36" s="42">
+        <v>4</v>
+      </c>
       <c r="M36" s="42"/>
       <c r="N36" s="42"/>
-      <c r="O36" s="42"/>
+      <c r="O36" s="42">
+        <v>8</v>
+      </c>
       <c r="P36" s="42"/>
       <c r="Q36" s="43"/>
       <c r="R36" s="72"/>
@@ -24293,16 +24400,32 @@
       <c r="C42" s="46"/>
       <c r="D42" s="41"/>
       <c r="E42" s="42"/>
-      <c r="F42" s="42"/>
-      <c r="G42" s="42"/>
-      <c r="H42" s="42"/>
-      <c r="I42" s="42"/>
-      <c r="J42" s="42"/>
-      <c r="K42" s="42"/>
-      <c r="L42" s="42"/>
+      <c r="F42" s="42">
+        <v>682</v>
+      </c>
+      <c r="G42" s="42">
+        <v>21</v>
+      </c>
+      <c r="H42" s="42">
+        <v>5</v>
+      </c>
+      <c r="I42" s="42">
+        <v>9</v>
+      </c>
+      <c r="J42" s="42">
+        <v>3</v>
+      </c>
+      <c r="K42" s="42">
+        <v>11</v>
+      </c>
+      <c r="L42" s="42">
+        <v>4</v>
+      </c>
       <c r="M42" s="42"/>
       <c r="N42" s="42"/>
-      <c r="O42" s="42"/>
+      <c r="O42" s="42">
+        <v>8</v>
+      </c>
       <c r="P42" s="42"/>
       <c r="Q42" s="43"/>
       <c r="R42" s="82" t="s">
@@ -24346,7 +24469,10 @@
       <c r="B44" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="90"/>
+      <c r="C44" s="90">
+        <f>1+8+1+1+1+71+3+644+5</f>
+        <v>735</v>
+      </c>
       <c r="D44" s="90"/>
       <c r="E44" s="90"/>
     </row>
@@ -24354,7 +24480,10 @@
       <c r="B45" s="76" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="90"/>
+      <c r="C45" s="90">
+        <f>4</f>
+        <v>4</v>
+      </c>
       <c r="D45" s="90"/>
       <c r="E45" s="90"/>
     </row>
@@ -24753,12 +24882,16 @@
     </row>
     <row r="8" spans="2:27" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="12"/>
-      <c r="C8" s="13"/>
+      <c r="C8" s="13" t="s">
+        <v>77</v>
+      </c>
       <c r="D8" s="14"/>
       <c r="E8" s="14"/>
       <c r="F8" s="14"/>
       <c r="G8" s="14"/>
-      <c r="H8" s="14"/>
+      <c r="H8" s="14" t="s">
+        <v>80</v>
+      </c>
       <c r="I8" s="14"/>
       <c r="J8" s="14"/>
       <c r="K8" s="14"/>
@@ -24768,14 +24901,22 @@
       <c r="O8" s="14"/>
       <c r="P8" s="14"/>
       <c r="Q8" s="14"/>
-      <c r="R8" s="14"/>
+      <c r="R8" s="14" t="s">
+        <v>81</v>
+      </c>
       <c r="S8" s="14"/>
-      <c r="T8" s="14"/>
+      <c r="T8" s="14" t="s">
+        <v>82</v>
+      </c>
       <c r="U8" s="14"/>
       <c r="V8" s="14"/>
-      <c r="W8" s="14"/>
+      <c r="W8" s="14" t="s">
+        <v>82</v>
+      </c>
       <c r="X8" s="59"/>
-      <c r="Y8" s="15"/>
+      <c r="Y8" s="15">
+        <v>1</v>
+      </c>
     </row>
     <row r="9" spans="2:27" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="12" t="s">
@@ -24941,12 +25082,16 @@
       <c r="B15" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="22"/>
+      <c r="C15" s="22" t="s">
+        <v>77</v>
+      </c>
       <c r="D15" s="23"/>
       <c r="E15" s="23"/>
       <c r="F15" s="23"/>
       <c r="G15" s="23"/>
-      <c r="H15" s="23"/>
+      <c r="H15" s="23" t="s">
+        <v>79</v>
+      </c>
       <c r="I15" s="23"/>
       <c r="J15" s="23"/>
       <c r="K15" s="23"/>
@@ -24956,25 +25101,37 @@
       <c r="O15" s="23"/>
       <c r="P15" s="23"/>
       <c r="Q15" s="23"/>
-      <c r="R15" s="23"/>
+      <c r="R15" s="23" t="s">
+        <v>81</v>
+      </c>
       <c r="S15" s="23"/>
-      <c r="T15" s="23"/>
+      <c r="T15" s="23">
+        <v>0</v>
+      </c>
       <c r="U15" s="23"/>
       <c r="V15" s="23"/>
-      <c r="W15" s="23"/>
+      <c r="W15" s="23">
+        <v>0</v>
+      </c>
       <c r="X15" s="61"/>
-      <c r="Y15" s="24"/>
+      <c r="Y15" s="24">
+        <v>0</v>
+      </c>
     </row>
     <row r="16" spans="2:27" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B16" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="C16" s="57"/>
+      <c r="C16" s="57">
+        <v>0</v>
+      </c>
       <c r="D16" s="58"/>
       <c r="E16" s="27"/>
       <c r="F16" s="27"/>
       <c r="G16" s="28"/>
-      <c r="H16" s="28"/>
+      <c r="H16" s="28" t="s">
+        <v>78</v>
+      </c>
       <c r="I16" s="28"/>
       <c r="J16" s="28"/>
       <c r="K16" s="56"/>
@@ -24984,14 +25141,22 @@
       <c r="O16" s="28"/>
       <c r="P16" s="28"/>
       <c r="Q16" s="28"/>
-      <c r="R16" s="28"/>
+      <c r="R16" s="28">
+        <v>0</v>
+      </c>
       <c r="S16" s="28"/>
-      <c r="T16" s="28"/>
+      <c r="T16" s="28" t="s">
+        <v>82</v>
+      </c>
       <c r="U16" s="28"/>
       <c r="V16" s="28"/>
-      <c r="W16" s="56"/>
+      <c r="W16" s="56" t="s">
+        <v>82</v>
+      </c>
       <c r="X16" s="62"/>
-      <c r="Y16" s="29"/>
+      <c r="Y16" s="29">
+        <v>1</v>
+      </c>
     </row>
     <row r="17" spans="2:25" s="5" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B17" s="30"/>
@@ -25393,17 +25558,29 @@
       <c r="C24" s="13"/>
       <c r="D24" s="14"/>
       <c r="E24" s="14"/>
-      <c r="F24" s="14"/>
+      <c r="F24" s="14">
+        <v>2</v>
+      </c>
       <c r="G24" s="14"/>
-      <c r="H24" s="14"/>
+      <c r="H24" s="14">
+        <v>2</v>
+      </c>
       <c r="I24" s="14"/>
       <c r="J24" s="14"/>
-      <c r="K24" s="14"/>
-      <c r="L24" s="14"/>
-      <c r="M24" s="14"/>
+      <c r="K24" s="14">
+        <v>71</v>
+      </c>
+      <c r="L24" s="14">
+        <v>18</v>
+      </c>
+      <c r="M24" s="14">
+        <v>432</v>
+      </c>
       <c r="N24" s="14"/>
       <c r="O24" s="14"/>
-      <c r="P24" s="14"/>
+      <c r="P24" s="14" t="s">
+        <v>83</v>
+      </c>
       <c r="Q24" s="14"/>
       <c r="R24" s="14"/>
       <c r="S24" s="14"/>
@@ -25579,17 +25756,29 @@
       <c r="C31" s="22"/>
       <c r="D31" s="23"/>
       <c r="E31" s="23"/>
-      <c r="F31" s="23"/>
+      <c r="F31" s="23">
+        <v>2</v>
+      </c>
       <c r="G31" s="23"/>
-      <c r="H31" s="23"/>
+      <c r="H31" s="23">
+        <v>0</v>
+      </c>
       <c r="I31" s="23"/>
       <c r="J31" s="23"/>
-      <c r="K31" s="23"/>
-      <c r="L31" s="23"/>
-      <c r="M31" s="23"/>
+      <c r="K31" s="23">
+        <v>1</v>
+      </c>
+      <c r="L31" s="23">
+        <v>5</v>
+      </c>
+      <c r="M31" s="23">
+        <v>93</v>
+      </c>
       <c r="N31" s="23"/>
       <c r="O31" s="23"/>
-      <c r="P31" s="23"/>
+      <c r="P31" s="23" t="s">
+        <v>83</v>
+      </c>
       <c r="Q31" s="23"/>
       <c r="R31" s="23"/>
       <c r="S31" s="23"/>
@@ -25607,17 +25796,29 @@
       <c r="C32" s="26"/>
       <c r="D32" s="27"/>
       <c r="E32" s="27"/>
-      <c r="F32" s="27"/>
+      <c r="F32" s="27">
+        <v>0</v>
+      </c>
       <c r="G32" s="28"/>
-      <c r="H32" s="28"/>
+      <c r="H32" s="28">
+        <v>2</v>
+      </c>
       <c r="I32" s="28"/>
       <c r="J32" s="28"/>
-      <c r="K32" s="28"/>
-      <c r="L32" s="28"/>
-      <c r="M32" s="28"/>
+      <c r="K32" s="28">
+        <v>70</v>
+      </c>
+      <c r="L32" s="28">
+        <v>13</v>
+      </c>
+      <c r="M32" s="28">
+        <v>339</v>
+      </c>
       <c r="N32" s="28"/>
       <c r="O32" s="23"/>
-      <c r="P32" s="28"/>
+      <c r="P32" s="28">
+        <v>0</v>
+      </c>
       <c r="Q32" s="28"/>
       <c r="R32" s="28"/>
       <c r="S32" s="28"/>
@@ -25757,17 +25958,29 @@
       <c r="C36" s="46"/>
       <c r="D36" s="41"/>
       <c r="E36" s="42"/>
-      <c r="F36" s="42"/>
-      <c r="G36" s="42"/>
+      <c r="F36" s="42">
+        <v>355</v>
+      </c>
+      <c r="G36" s="42">
+        <v>1</v>
+      </c>
       <c r="H36" s="42"/>
-      <c r="I36" s="42"/>
+      <c r="I36" s="42">
+        <v>5</v>
+      </c>
       <c r="J36" s="42"/>
       <c r="K36" s="42"/>
-      <c r="L36" s="42"/>
+      <c r="L36" s="42">
+        <v>83</v>
+      </c>
       <c r="M36" s="42"/>
       <c r="N36" s="42"/>
-      <c r="O36" s="42"/>
-      <c r="P36" s="42"/>
+      <c r="O36" s="42">
+        <v>2</v>
+      </c>
+      <c r="P36" s="42">
+        <v>6</v>
+      </c>
       <c r="Q36" s="43"/>
       <c r="R36" s="72"/>
       <c r="S36" s="44"/>
@@ -25915,17 +26128,29 @@
       <c r="C42" s="46"/>
       <c r="D42" s="41"/>
       <c r="E42" s="42"/>
-      <c r="F42" s="42"/>
-      <c r="G42" s="42"/>
+      <c r="F42" s="42">
+        <v>355</v>
+      </c>
+      <c r="G42" s="42">
+        <v>1</v>
+      </c>
       <c r="H42" s="42"/>
-      <c r="I42" s="42"/>
+      <c r="I42" s="42">
+        <v>5</v>
+      </c>
       <c r="J42" s="42"/>
       <c r="K42" s="42"/>
-      <c r="L42" s="42"/>
+      <c r="L42" s="42">
+        <v>83</v>
+      </c>
       <c r="M42" s="42"/>
       <c r="N42" s="42"/>
-      <c r="O42" s="42"/>
-      <c r="P42" s="42"/>
+      <c r="O42" s="42">
+        <v>2</v>
+      </c>
+      <c r="P42" s="42">
+        <v>6</v>
+      </c>
       <c r="Q42" s="43"/>
       <c r="R42" s="82" t="s">
         <v>54</v>
@@ -26006,7 +26231,8 @@
   <cols>
     <col min="1" max="1" width="1.140625" style="2" customWidth="1"/>
     <col min="2" max="2" width="14.42578125" style="2" customWidth="1"/>
-    <col min="3" max="8" width="5.7109375" style="2" customWidth="1"/>
+    <col min="3" max="7" width="5.7109375" style="2" customWidth="1"/>
+    <col min="8" max="8" width="7" style="2" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="8" style="2" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="7" style="2" bestFit="1" customWidth="1"/>
     <col min="11" max="13" width="5.7109375" style="2" customWidth="1"/>
@@ -26375,12 +26601,16 @@
     </row>
     <row r="8" spans="2:27" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="12"/>
-      <c r="C8" s="13"/>
+      <c r="C8" s="13">
+        <v>2</v>
+      </c>
       <c r="D8" s="14"/>
       <c r="E8" s="14"/>
       <c r="F8" s="14"/>
       <c r="G8" s="14"/>
-      <c r="H8" s="14"/>
+      <c r="H8" s="14" t="s">
+        <v>86</v>
+      </c>
       <c r="I8" s="14"/>
       <c r="J8" s="14"/>
       <c r="K8" s="14"/>
@@ -26390,14 +26620,22 @@
       <c r="O8" s="14"/>
       <c r="P8" s="14"/>
       <c r="Q8" s="14"/>
-      <c r="R8" s="14"/>
+      <c r="R8" s="14">
+        <v>2</v>
+      </c>
       <c r="S8" s="14"/>
-      <c r="T8" s="14"/>
+      <c r="T8" s="14">
+        <v>2</v>
+      </c>
       <c r="U8" s="14"/>
       <c r="V8" s="14"/>
-      <c r="W8" s="14"/>
+      <c r="W8" s="14">
+        <v>4</v>
+      </c>
       <c r="X8" s="59"/>
-      <c r="Y8" s="15"/>
+      <c r="Y8" s="15">
+        <v>1</v>
+      </c>
     </row>
     <row r="9" spans="2:27" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="12" t="s">
@@ -26563,12 +26801,16 @@
       <c r="B15" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="22"/>
+      <c r="C15" s="22">
+        <v>2</v>
+      </c>
       <c r="D15" s="23"/>
       <c r="E15" s="23"/>
       <c r="F15" s="23"/>
       <c r="G15" s="23"/>
-      <c r="H15" s="23"/>
+      <c r="H15" s="23" t="s">
+        <v>85</v>
+      </c>
       <c r="I15" s="23"/>
       <c r="J15" s="23"/>
       <c r="K15" s="23"/>
@@ -26578,25 +26820,37 @@
       <c r="O15" s="23"/>
       <c r="P15" s="23"/>
       <c r="Q15" s="23"/>
-      <c r="R15" s="23"/>
+      <c r="R15" s="23">
+        <v>2</v>
+      </c>
       <c r="S15" s="23"/>
-      <c r="T15" s="23"/>
+      <c r="T15" s="23">
+        <v>0</v>
+      </c>
       <c r="U15" s="23"/>
       <c r="V15" s="23"/>
-      <c r="W15" s="23"/>
+      <c r="W15" s="23">
+        <v>1</v>
+      </c>
       <c r="X15" s="61"/>
-      <c r="Y15" s="24"/>
+      <c r="Y15" s="24">
+        <v>1</v>
+      </c>
     </row>
     <row r="16" spans="2:27" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B16" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="C16" s="57"/>
+      <c r="C16" s="57">
+        <v>0</v>
+      </c>
       <c r="D16" s="58"/>
       <c r="E16" s="27"/>
       <c r="F16" s="27"/>
       <c r="G16" s="28"/>
-      <c r="H16" s="28"/>
+      <c r="H16" s="28" t="s">
+        <v>84</v>
+      </c>
       <c r="I16" s="28"/>
       <c r="J16" s="28"/>
       <c r="K16" s="56"/>
@@ -26606,14 +26860,22 @@
       <c r="O16" s="28"/>
       <c r="P16" s="28"/>
       <c r="Q16" s="28"/>
-      <c r="R16" s="28"/>
+      <c r="R16" s="28">
+        <v>0</v>
+      </c>
       <c r="S16" s="28"/>
-      <c r="T16" s="28"/>
+      <c r="T16" s="28">
+        <v>2</v>
+      </c>
       <c r="U16" s="28"/>
       <c r="V16" s="28"/>
-      <c r="W16" s="56"/>
+      <c r="W16" s="56">
+        <v>3</v>
+      </c>
       <c r="X16" s="62"/>
-      <c r="Y16" s="29"/>
+      <c r="Y16" s="29">
+        <v>0</v>
+      </c>
     </row>
     <row r="17" spans="2:25" s="5" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B17" s="30"/>
@@ -27015,17 +27277,29 @@
       <c r="C24" s="13"/>
       <c r="D24" s="14"/>
       <c r="E24" s="14"/>
-      <c r="F24" s="14"/>
+      <c r="F24" s="14">
+        <v>2</v>
+      </c>
       <c r="G24" s="14"/>
-      <c r="H24" s="14"/>
+      <c r="H24" s="14">
+        <v>112</v>
+      </c>
       <c r="I24" s="14"/>
       <c r="J24" s="14"/>
-      <c r="K24" s="14"/>
-      <c r="L24" s="14"/>
-      <c r="M24" s="14"/>
+      <c r="K24" s="14">
+        <v>2</v>
+      </c>
+      <c r="L24" s="14">
+        <v>17</v>
+      </c>
+      <c r="M24" s="14">
+        <v>598</v>
+      </c>
       <c r="N24" s="14"/>
       <c r="O24" s="14"/>
-      <c r="P24" s="14"/>
+      <c r="P24" s="14">
+        <v>8</v>
+      </c>
       <c r="Q24" s="14"/>
       <c r="R24" s="14"/>
       <c r="S24" s="14"/>
@@ -27201,17 +27475,29 @@
       <c r="C31" s="22"/>
       <c r="D31" s="23"/>
       <c r="E31" s="23"/>
-      <c r="F31" s="23"/>
+      <c r="F31" s="23">
+        <v>2</v>
+      </c>
       <c r="G31" s="23"/>
-      <c r="H31" s="23"/>
+      <c r="H31" s="23">
+        <v>77</v>
+      </c>
       <c r="I31" s="23"/>
       <c r="J31" s="23"/>
-      <c r="K31" s="23"/>
-      <c r="L31" s="23"/>
-      <c r="M31" s="23"/>
+      <c r="K31" s="23">
+        <v>0</v>
+      </c>
+      <c r="L31" s="23">
+        <v>0</v>
+      </c>
+      <c r="M31" s="23">
+        <v>116</v>
+      </c>
       <c r="N31" s="23"/>
       <c r="O31" s="23"/>
-      <c r="P31" s="23"/>
+      <c r="P31" s="23">
+        <v>8</v>
+      </c>
       <c r="Q31" s="23"/>
       <c r="R31" s="23"/>
       <c r="S31" s="23"/>
@@ -27229,17 +27515,29 @@
       <c r="C32" s="26"/>
       <c r="D32" s="27"/>
       <c r="E32" s="27"/>
-      <c r="F32" s="27"/>
+      <c r="F32" s="27">
+        <v>0</v>
+      </c>
       <c r="G32" s="28"/>
-      <c r="H32" s="28"/>
+      <c r="H32" s="28">
+        <v>35</v>
+      </c>
       <c r="I32" s="28"/>
       <c r="J32" s="28"/>
-      <c r="K32" s="28"/>
-      <c r="L32" s="28"/>
-      <c r="M32" s="28"/>
+      <c r="K32" s="28">
+        <v>2</v>
+      </c>
+      <c r="L32" s="28">
+        <v>17</v>
+      </c>
+      <c r="M32" s="28">
+        <v>482</v>
+      </c>
       <c r="N32" s="28"/>
       <c r="O32" s="23"/>
-      <c r="P32" s="28"/>
+      <c r="P32" s="28">
+        <v>0</v>
+      </c>
       <c r="Q32" s="28"/>
       <c r="R32" s="28"/>
       <c r="S32" s="28"/>
@@ -27378,19 +27676,41 @@
       </c>
       <c r="C36" s="46"/>
       <c r="D36" s="41"/>
-      <c r="E36" s="42"/>
-      <c r="F36" s="42"/>
-      <c r="G36" s="42"/>
+      <c r="E36" s="42">
+        <v>2</v>
+      </c>
+      <c r="F36" s="42">
+        <v>577</v>
+      </c>
+      <c r="G36" s="42">
+        <v>7</v>
+      </c>
       <c r="H36" s="42"/>
-      <c r="I36" s="42"/>
-      <c r="J36" s="42"/>
-      <c r="K36" s="42"/>
-      <c r="L36" s="42"/>
-      <c r="M36" s="42"/>
-      <c r="N36" s="42"/>
-      <c r="O36" s="42"/>
+      <c r="I36" s="42">
+        <v>4</v>
+      </c>
+      <c r="J36" s="42">
+        <v>2</v>
+      </c>
+      <c r="K36" s="42">
+        <v>7</v>
+      </c>
+      <c r="L36" s="42">
+        <v>3</v>
+      </c>
+      <c r="M36" s="42">
+        <v>4</v>
+      </c>
+      <c r="N36" s="42">
+        <v>19</v>
+      </c>
+      <c r="O36" s="42">
+        <v>12</v>
+      </c>
       <c r="P36" s="42"/>
-      <c r="Q36" s="43"/>
+      <c r="Q36" s="43">
+        <v>39</v>
+      </c>
       <c r="R36" s="72"/>
       <c r="S36" s="44"/>
       <c r="T36" s="44"/>
@@ -27536,19 +27856,41 @@
       </c>
       <c r="C42" s="46"/>
       <c r="D42" s="41"/>
-      <c r="E42" s="42"/>
-      <c r="F42" s="42"/>
-      <c r="G42" s="42"/>
+      <c r="E42" s="42">
+        <v>2</v>
+      </c>
+      <c r="F42" s="42">
+        <v>577</v>
+      </c>
+      <c r="G42" s="42">
+        <v>7</v>
+      </c>
       <c r="H42" s="42"/>
-      <c r="I42" s="42"/>
-      <c r="J42" s="42"/>
-      <c r="K42" s="42"/>
-      <c r="L42" s="42"/>
-      <c r="M42" s="42"/>
-      <c r="N42" s="42"/>
-      <c r="O42" s="42"/>
+      <c r="I42" s="42">
+        <v>4</v>
+      </c>
+      <c r="J42" s="42">
+        <v>2</v>
+      </c>
+      <c r="K42" s="42">
+        <v>7</v>
+      </c>
+      <c r="L42" s="42">
+        <v>3</v>
+      </c>
+      <c r="M42" s="42">
+        <v>4</v>
+      </c>
+      <c r="N42" s="42">
+        <v>19</v>
+      </c>
+      <c r="O42" s="42">
+        <v>12</v>
+      </c>
       <c r="P42" s="42"/>
-      <c r="Q42" s="43"/>
+      <c r="Q42" s="43">
+        <v>39</v>
+      </c>
       <c r="R42" s="82" t="s">
         <v>54</v>
       </c>
@@ -27590,7 +27932,10 @@
       <c r="B44" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="90"/>
+      <c r="C44" s="90">
+        <f>21+2+3+35+2+17+482</f>
+        <v>562</v>
+      </c>
       <c r="D44" s="90"/>
       <c r="E44" s="90"/>
     </row>
@@ -27598,7 +27943,10 @@
       <c r="B45" s="76" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="90"/>
+      <c r="C45" s="90">
+        <f>22</f>
+        <v>22</v>
+      </c>
       <c r="D45" s="90"/>
       <c r="E45" s="90"/>
     </row>

</xml_diff>